<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-11 Le chemin d'escargot de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-11.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-11.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le chemin d'argent de Sarah</t>
+          <t>Le chemin d'escargot de Sarah</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>allée, classe, coin des livres</t>
+          <t>entrée au radiateur, classe, tapis, coin des livres</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, papa, maman, maîtresse</t>
+          <t>Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut raconter le chemin d'escargot sur la boîte aux lettres, puis le livre. Elle lève la main, elle attend, puis elle parle.</t>
+          <t>Un chemin d'argent court sur la vitre. Sur le chemin, un éclat d'escargot brille. Sarah veut le dire, maintenant. Elle coupe papa : les mots se perdent. À la classe, elle ouvre la bouche trop tôt. Elle refuse de foncer, lève la main, attend, parle. Merci vécu. L'éclat d'escargot tient sur la vitre.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un bouton de laine pend au manteau. Il tient par un seul fil, tout fin. L'écharpe chatouille encore la joue de Sarah. Elle sent le savon de maman. L'écharpe, un tour. Pas trop serré. Tes gants sont dans la poche. Tu les sens ? Oui. Ils sont tout doux. Dehors, l'air est frais et calme. Sur la boîte aux lettres, une traînée brillante. Un escargot est passé, tout lentement. Tu as vu le petit chemin luisant ? Il brille. Comme un fil d'argent. Tu pourras le raconter. Le chemin sent l'herbe coupée. La classe sent les crayons et le lait tiède. Au revoir, Sarah. On revient. Au revoir, maman. Tu poses l'écharpe au crochet. En ce moment, Sarah s'assoit près de la fenêtre. Elle pose les mains sur ses genoux. Une autre traînée brille un peu sur la vitre. Bonjour. Bonjour. Qui a vu un petit animal tout lent ? Sarah a une idée. L'escargot de la boîte aux lettres. Le chemin d'argent. Le mot est déjà là. Elle avance un peu sur sa chaise. La maîtresse range encore des crayons dans un pot. Le pot fait un petit bruit de bois.</t>
+          <t>Un chemin d'argent court sur la vitre. Il est mince, un peu luisant. L'air sent le savon de maman. L'écharpe de laine chatouille la joue de Sarah. Elle pique un peu, maman. C'est la laine, près du cou. Le radiateur de l'entrée fait tic. Tu l'entends, Sarah ? Oui, papa. Il chante, près de nous. Sarah connaît cette entrée. Ce chemin, lui, est nouveau. Sur la vitre, un éclat d'escargot brille. Il est petit, papa. C'est le soleil sur le chemin. Un escargot est passé ! Tu as vu le petit chemin luisant ? Il brille. Je veux le dire, maintenant ! Tes gants sont dans la poche. Tu les sens ? Oui. Ils sont chauds. Dehors, l'air est frais. La vitre est froide sous le doigt. Elle est lisse, papa. Maman tourne l'écharpe, un tour. Pas trop serré. D'accord, maman. Papa parle près du crochet. L'écharpe, au crochet, Sarah. Les mots de Sarah se cognent aux siens. Personne ne tourne la tête. Papa, le chemin ! Tu disais quelque chose, Sarah ? Le chemin d'argent. Le sourire de Sarah disparaît. L'éclat d'escargot tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux raconter le chemin ? Oui, papa. Tu vas t'asseoir sur le tapis ? D'accord, maman. Au revoir, Sarah. Au revoir, maman. On revient te chercher. Au revoir, papa. En ce moment, Sarah entre dans la classe. La classe sent les crayons et le lait tiède. Sarah pose l'écharpe au crochet. Le tapis est un peu froid, sous les genoux. Elle s'assoit près de la fenêtre. Elle pose les mains sur ses genoux. Le chemin d'argent reste sur la vitre. La maîtresse parle près du tapis. Une affiche montre un animal lent. Sarah a une idée. Le chemin d'escargot brille, près d'elle. Je veux parler du chemin.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un bouton de laine pend au manteau. Il tient par un seul fil, tout fin. L'écharpe chatouille encore la joue de Sarah. Elle sent le savon de maman. L'écharpe, un tour. Pas trop serré. Tes gants sont dans la poche. Tu les sens ? Oui. Ils sont tout doux. Dehors, l'air est frais et calme. Sur la boîte aux lettres, une traînée brillante. Un escargot est passé, tout lentement. Tu as vu le petit chemin luisant ? Il brille. Comme un fil d'argent. Tu pourras le raconter. Le chemin sent l'herbe coupée. La classe sent les crayons et le lait tiède. Au revoir, Sarah. On revient. Au revoir, maman. Tu poses l'écharpe au crochet. En ce moment, Sarah s'assoit près de la fenêtre. Elle pose les mains sur ses genoux. Une autre traînée brille un peu sur la vitre. Bonjour. Bonjour. Qui a vu un petit animal tout lent ? Sarah a une idée. L'escargot de la boîte aux lettres. Le chemin d'argent. Le mot est déjà là. Elle avance un peu sur sa chaise. La maîtresse range encore des crayons dans un pot. Le pot fait un petit bruit de bois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un chemin d'argent court sur la vitre. Il est mince, un peu luisant. L'air sent le savon de maman. L'écharpe de laine chatouille la joue de Sarah. Elle pique un peu, maman. C'est la laine, près du cou. Le radiateur de l'entrée fait tic. Tu l'entends, Sarah ? Oui, papa. Il chante, près de nous. Sarah connaît cette entrée. Ce chemin, lui, est nouveau. Sur la vitre, un &lt;emphasis level="moderate"&gt;éclat d'escargot&lt;/emphasis&gt; brille. Il est petit, papa. C'est le soleil sur le chemin. Un escargot est passé ! Tu as vu le petit chemin luisant ? Il brille. Je veux le dire, maintenant ! Tes gants sont dans la poche. Tu les sens ? Oui. Ils sont chauds. Dehors, l'air est frais. La vitre est froide sous le doigt. Elle est lisse, papa. Maman tourne l'écharpe, un tour. Pas trop serré. D'accord, maman. Papa parle près du crochet. L'écharpe, au crochet, Sarah. Les mots de Sarah se cognent aux siens. Personne ne tourne la tête. Papa, le chemin ! Tu disais quelque chose, Sarah ? Le chemin d'argent. Le sourire de Sarah disparaît. L'éclat d'escargot tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux raconter le chemin ? Oui, papa. Tu vas t'asseoir sur le tapis ? D'accord, maman. Au revoir, Sarah. Au revoir, maman. On revient te chercher. Au revoir, papa. En ce moment, Sarah entre dans la classe. La classe sent les crayons et le lait tiède. Sarah pose l'écharpe au crochet. Le tapis est un peu froid, sous les genoux. Elle s'assoit près de la fenêtre. Elle pose les mains sur ses genoux. Le chemin d'argent reste sur la vitre. La maîtresse parle près du tapis. Une affiche montre un animal lent. Sarah a une idée. Le chemin d'escargot brille, près d'elle. Je veux parler du chemin.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Francine arrive en classe avec maman. Maman dit au revoir. Francine s'assoit sur le tapis. La maîtresse pose une question. Francine a une idée. Elle lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Francine attend encore. Puis la maîtresse dit : Francine, c'est ton tour. Francine parle. Elle dit : le nuage est blanc. La maîtresse sourit. Plus tard, au coin des livres, Francine a encore une idée. Même leçon, autre lieu. Elle lève la main. Elle attend. Puis parler, c'est son tour. Elle dit : j'aime ce livre. Le soir, maman demande. Francine dit : j'ai levé la main. J'ai su attendre. Puis parler, c'était mon tour. [pause]</t>
+          <t>Un chemin d'argent court sur la vitre. Il est mince, un peu luisant. L'air sent le savon de maman. L'écharpe de laine chatouille la joue de Sarah. Elle pique un peu, maman. C'est la laine, près du cou. Le radiateur de l'entrée fait tic. Tu l'entends, Sarah ? Oui, papa. Il chante, près de nous. Sarah connaît cette entrée. Ce chemin, lui, est nouveau. Sur la vitre, un &lt;emphasis&gt;éclat d'escargot&lt;/emphasis&gt; brille. Il est petit, papa. C'est le soleil sur le chemin. Un escargot est passé ! Tu as vu le petit chemin luisant ? Il brille. Je veux le dire, maintenant ! Tes gants sont dans la poche. Tu les sens ? Oui. Ils sont chauds. Dehors, l'air est frais. La vitre est froide sous le doigt. Elle est lisse, papa. Maman tourne l'écharpe, un tour. Pas trop serré. D'accord, maman. Papa parle près du crochet. L'écharpe, au crochet, Sarah. Les mots de Sarah se cognent aux siens. Personne ne tourne la tête. Papa, le chemin ! Tu disais quelque chose, Sarah ? Le chemin d'argent. Le sourire de Sarah disparaît. L'éclat d'escargot tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux raconter le chemin ? Oui, papa. Tu vas t'asseoir sur le tapis ? D'accord, maman. Au revoir, Sarah. Au revoir, maman. On revient te chercher. Au revoir, papa. En ce moment, Sarah entre dans la classe. La classe sent les crayons et le lait tiède. Sarah pose l'écharpe au crochet. Le tapis est un peu froid, sous les genoux. Elle s'assoit près de la fenêtre. Elle pose les mains sur ses genoux. Le chemin d'argent reste sur la vitre. La maîtresse parle près du tapis. Une affiche montre un animal lent. Sarah a une idée. Le chemin d'escargot brille, près d'elle. Je veux parler du chemin. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat d'escargot</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,50 +1326,80 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_dire_le_chemin_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un bouton de laine pend au manteau.
-narrateur|Il tient par un seul fil, tout fin.
-narrateur|L'écharpe chatouille encore la joue de Sarah.
-narrateur|Elle sent le savon de maman.
-maman|L'écharpe, un tour.
-maman|Pas trop serré.
+          <t>narrateur|Un chemin d'argent court sur la vitre.
+narrateur|Il est mince, un peu luisant.
+narrateur|L'air sent le savon de maman.
+narrateur|L'écharpe de laine chatouille la joue de Sarah.
+enfant-f|Elle pique un peu, maman.
+maman|C'est la laine, près du cou.
+papa|Le radiateur de l'entrée fait tic.
+papa|Tu l'entends, Sarah ?
+enfant-f|Oui, papa.
+enfant-f|Il chante, près de nous.
+narrateur|Sarah connaît cette entrée.
+narrateur|Ce chemin, lui, est nouveau.
+narrateur|Sur la vitre, un éclat d'escargot brille.
+enfant-f|Il est petit, papa.
+papa|C'est le soleil sur le chemin.
+enfant-f|Un escargot est passé !
+maman|Tu as vu le petit chemin luisant ?
+enfant-f|Il brille.
+enfant-f|Je veux le dire, maintenant !
 papa|Tes gants sont dans la poche.
 papa|Tu les sens ?
 enfant-f|Oui.
-enfant-f|Ils sont tout doux.
-narrateur|Dehors, l'air est frais et calme.
-narrateur|Sur la boîte aux lettres, une traînée brillante.
-narrateur|Un escargot est passé, tout lentement.
-papa|Tu as vu le petit chemin luisant ?
-enfant-f|Il brille.
-enfant-f|Comme un fil d'argent.
-maman|Tu pourras le raconter.
-narrateur|Le chemin sent l'herbe coupée.
+enfant-f|Ils sont chauds.
+narrateur|Dehors, l'air est frais.
+narrateur|La vitre est froide sous le doigt.
+enfant-f|Elle est lisse, papa.
+narrateur|Maman tourne l'écharpe, un tour.
+maman|Pas trop serré.
+enfant-f|D'accord, maman.
+narrateur|Papa parle près du crochet.
+papa|L'écharpe, au crochet, Sarah.
+narrateur|Les mots de Sarah se cognent aux siens.
+narrateur|Personne ne tourne la tête.
+enfant-f|Papa, le chemin !
+papa|Tu disais quelque chose, Sarah ?
+enfant-f|Le chemin d'argent.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|L'éclat d'escargot tremble, puis tient.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Ça ne sort pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu veux raconter le chemin ?
+enfant-f|Oui, papa.
+maman|Tu vas t'asseoir sur le tapis ?
+enfant-f|D'accord, maman.
+maman|Au revoir, Sarah.
+enfant-f|Au revoir, maman.
+papa|On revient te chercher.
+enfant-f|Au revoir, papa.
+narrateur|En ce moment, Sarah entre dans la classe.
 narrateur|La classe sent les crayons et le lait tiède.
-maman|Au revoir, Sarah.
-maman|On revient.
-enfant-f|Au revoir, maman.
-papa|Tu poses l'écharpe au crochet.
-narrateur|En ce moment, Sarah s'assoit près de la fenêtre.
+narrateur|Sarah pose l'écharpe au crochet.
+narrateur|Le tapis est un peu froid, sous les genoux.
+narrateur|Elle s'assoit près de la fenêtre.
 narrateur|Elle pose les mains sur ses genoux.
-narrateur|Une autre traînée brille un peu sur la vitre.
-maitresse|Bonjour.
-enfant-f|Bonjour.
-maitresse|Qui a vu un petit animal tout lent ?
+narrateur|Le chemin d'argent reste sur la vitre.
+narrateur|La maîtresse parle près du tapis.
+narrateur|Une affiche montre un animal lent.
 narrateur|Sarah a une idée.
-narrateur|L'escargot de la boîte aux lettres.
-narrateur|Le chemin d'argent.
-narrateur|Le mot est déjà là.
-narrateur|Elle avance un peu sur sa chaise.
-narrateur|La maîtresse range encore des crayons dans un pot.
-narrateur|Le pot fait un petit bruit de bois.</t>
+narrateur|Le chemin d'escargot brille, près d'elle.
+enfant-f|Je veux parler du chemin.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>radiateur,echarpe</t>
         </is>
       </c>
     </row>
@@ -1401,12 +1431,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-elle d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Francine veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-elle d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1469,18 +1499,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1495,34 +1525,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1531,23 +1565,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_attend_puis_parle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1580,17 +1614,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah lève la main. Elle attend, la main haute. Elle regarde la vitre, tout doucement. Sa main ne descend pas. Sarah, c'est toi. Tu peux parler. L'escargot a laissé un chemin. Il brille sur la boîte aux lettres. Comme un fil d'argent. Un chemin d'argent, oui. Il allait tout lentement. Merci, Sarah. Plus tard, au coin des livres, un banc de bois attend. Sarah ouvre un album aux pages épaisses. Il y a un escargot, tout lent, sur une feuille. Elle a encore une idée. Elle lève la main. Elle attend. Sarah, c'est toi, ici aussi. J'aime ce livre. Il y a un escargot, tout lent. Comme celui de la boîte. Comme celui de la boîte.</t>
+          <t>Sarah ouvre la bouche trop vite. L'escargot a laissé un chemin ! Un camarade parle, près du tapis. J'ai vu un ver de terre. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Sarah attend que le silence arrive. Sur la vitre, l'éclat d'escargot brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Un escargot a laissé un chemin. Il brille sur la vitre. Sarah montre la vitre du doigt. Il est mince, comme ça. Les genoux restent sur le tapis. Plus tard, c'est le coin des livres. Un banc de bois attend. Sarah ouvre un album aux pages épaisses. Sur une page, un escargot avance. Comme sur la vitre ! Sarah a envie de le dire, d'un coup.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah lève la main. Elle attend, la main haute. Elle regarde la vitre, tout doucement. Sa main ne descend pas. Sarah, c'est toi. Tu peux parler. L'escargot a laissé un chemin. Il brille sur la boîte aux lettres. Comme un fil d'argent. Un chemin d'argent, oui. Il allait tout lentement. Merci, Sarah. Plus tard, au coin des livres, un banc de bois attend. Sarah ouvre un album aux pages épaisses. Il y a un escargot, tout lent, sur une feuille. Elle a encore une idée. Elle lève la main. Elle attend. Sarah, c'est toi, ici aussi. J'aime ce livre. Il y a un escargot, tout lent. Comme celui de la boîte. Comme celui de la boîte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah ouvre la bouche trop vite. L'escargot a laissé un chemin ! Un camarade parle, près du tapis. J'ai vu un ver de terre. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Sarah attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Sur la vitre, l'éclat d'escargot brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Un escargot a laissé un chemin. Il brille sur la vitre. Sarah montre la vitre du doigt. Il est mince, comme ça. Les genoux restent sur le tapis. Plus tard, c'est le coin des livres. Un banc de bois attend. Sarah ouvre un album aux pages épaisses. Sur une page, un escargot avance. Comme sur la vitre ! Sarah a envie de le dire, d'un coup.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Francine a levé la main. Elle a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; parler, c'était son tour. Au tapis, puis aux livres. [pause]</t>
+          <t>Sarah ouvre la bouche trop vite. L'escargot a laissé un chemin ! Un camarade parle, près du tapis. J'ai vu un ver de terre. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Sarah attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Sur la vitre, l'éclat d'escargot brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Un escargot a laissé un chemin. Il brille sur la vitre. Sarah montre la vitre du doigt. Il est mince, comme ça. Les genoux restent sur le tapis. Plus tard, c'est le coin des livres. Un banc de bois attend. Sarah ouvre un album aux pages épaisses. Sur une page, un escargot avance. Comme sur la vitre ! Sarah a envie de le dire, d'un coup. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1637,7 +1671,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1645,10 +1679,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1671,7 +1705,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>silence</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1685,16 +1719,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1703,10 +1737,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1719,39 +1753,43 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=elle_refuse_de_foncer_puis_parle; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah lève la main.
-narrateur|Elle attend, la main haute.
-narrateur|Elle regarde la vitre, tout doucement.
-narrateur|Sa main ne descend pas.
-maitresse|Sarah, c'est toi.
-maitresse|Tu peux parler.
-enfant-f|L'escargot a laissé un chemin.
-enfant-f|Il brille sur la boîte aux lettres.
-enfant-f|Comme un fil d'argent.
-maitresse|Un chemin d'argent, oui.
-enfant-f|Il allait tout lentement.
-maitresse|Merci, Sarah.
-narrateur|Plus tard, au coin des livres, un banc de bois attend.
+          <t>narrateur|Sarah ouvre la bouche trop vite.
+enfant-f|L'escargot a laissé un chemin !
+narrateur|Un camarade parle, près du tapis.
+copain|J'ai vu un ver de terre.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Elle lève la main, près du tapis.
+narrateur|Sa main reste en l'air.
+narrateur|Le camarade finit sa phrase.
+narrateur|Sarah attend que le silence arrive.
+narrateur|Sur la vitre, l'éclat d'escargot brille.
+enfant-f|Je peux dire quelque chose ?
+narrateur|La classe tourne un peu la tête.
+enfant-f|Un escargot a laissé un chemin.
+enfant-f|Il brille sur la vitre.
+narrateur|Sarah montre la vitre du doigt.
+enfant-f|Il est mince, comme ça.
+narrateur|Les genoux restent sur le tapis.
+narrateur|Plus tard, c'est le coin des livres.
+narrateur|Un banc de bois attend.
 narrateur|Sarah ouvre un album aux pages épaisses.
-narrateur|Il y a un escargot, tout lent, sur une feuille.
-narrateur|Elle a encore une idée.
-narrateur|Elle lève la main.
-narrateur|Elle attend.
-maitresse|Sarah, c'est toi, ici aussi.
-enfant-f|J'aime ce livre.
-enfant-f|Il y a un escargot, tout lent.
-maitresse|Comme celui de la boîte.
-enfant-f|Comme celui de la boîte.</t>
+narrateur|Sur une page, un escargot avance.
+enfant-f|Comme sur la vitre !
+narrateur|Sarah a envie de le dire, d'un coup.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>pages</t>
+          <t>tapis,pages</t>
         </is>
       </c>
     </row>
@@ -1778,17 +1816,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Sarah range son cartable. L'écharpe de laine est encore au crochet. La porte s'ouvre. Tu as passé un bon moment ? J'ai parlé de l'escargot. Et du livre, aussi. Le chemin d'argent ? Oui. Sur la boîte aux lettres. On rentre. Le bouton tient encore, tout juste. Le soir, l'écharpe sèche près du radiateur. Sarah regarde la boîte aux lettres, par la porte. Le chemin est encore un peu là. Un peu, oui. Demain, il sera peut-être parti. Sarah touche le fil du bouton. On le recoud tout à l'heure. Le livre aussi avait un escargot. Tout lent, comme le vrai.</t>
+          <t>Sarah veut tout dire, d'un coup. Elle tire l'album trop vite. Les pages se collent un peu. L'album glisse vers le banc. Ça tombe ! Sarah veut foncer, d'un coup. Sarah refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle pose l'album à plat. Elle écoute le coin des livres. Un autre enfant feuillette, plus loin. Sarah attend le silence, un instant. Je peux dire quelque chose ? Il y a un escargot, dans le livre. La page sent le papier épais. Le soir, la porte s'ouvre. Te voilà, Sarah. L'écharpe sent le savon. Sarah pose le cartable contre le mur. J'ai parlé du chemin. Après le ver de terre. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre. L'écharpe, tu la vois ? Oui, papa. Le bois du crochet tient la laine.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Sarah range son cartable. L'écharpe de laine est encore au crochet. La porte s'ouvre. Tu as passé un bon moment ? J'ai parlé de l'escargot. Et du livre, aussi. Le chemin d'argent ? Oui. Sur la boîte aux lettres. On rentre. Le bouton tient encore, tout juste. Le soir, l'écharpe sèche près du radiateur. Sarah regarde la boîte aux lettres, par la porte. Le chemin est encore un peu là. Un peu, oui. Demain, il sera peut-être parti. Sarah touche le fil du bouton. On le recoud tout à l'heure. Le livre aussi avait un escargot. Tout lent, comme le vrai.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut tout dire, d'un coup. Elle tire l'&lt;emphasis level="moderate"&gt;album&lt;/emphasis&gt; trop vite. Les pages se collent un peu. L'album glisse vers le banc. Ça tombe ! Sarah veut foncer, d'un coup. Sarah refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle pose l'album à plat. Elle écoute le coin des livres. Un autre enfant feuillette, plus loin. Sarah attend le silence, un instant. Je peux dire quelque chose ? Il y a un escargot, dans le livre. La page sent le papier épais. Le soir, la porte s'ouvre. Te voilà, Sarah. L'écharpe sent le savon. Sarah pose le cartable contre le mur. J'ai parlé du chemin. Après le ver de terre. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre. L'écharpe, tu la vois ? Oui, papa. Le bois du crochet tient la laine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Francine range son cartable. Maman l'attend à la porte. [pause]</t>
+          <t>Sarah veut tout dire, d'un coup. Elle tire l'&lt;emphasis&gt;album&lt;/emphasis&gt; trop vite. Les pages se collent un peu. L'album glisse vers le banc. Ça tombe ! Sarah veut foncer, d'un coup. Sarah refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle pose l'album à plat. Elle écoute le coin des livres. Un autre enfant feuillette, plus loin. Sarah attend le silence, un instant. Je peux dire quelque chose ? Il y a un escargot, dans le livre. La page sent le papier épais. Le soir, la porte s'ouvre. Te voilà, Sarah. L'écharpe sent le savon. Sarah pose le cartable contre le mur. J'ai parlé du chemin. Après le ver de terre. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre. L'écharpe, tu la vois ? Oui, papa. Le bois du crochet tient la laine. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1835,7 +1873,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1843,10 +1881,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,28 +1905,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>album</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1897,10 +1939,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1911,34 +1953,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_l_eclat_tient; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Sarah range son cartable.
-narrateur|L'écharpe de laine est encore au crochet.
-narrateur|La porte s'ouvre.
-maman|Tu as passé un bon moment ?
-enfant-f|J'ai parlé de l'escargot.
-enfant-f|Et du livre, aussi.
-papa|Le chemin d'argent ?
-enfant-f|Oui.
-enfant-f|Sur la boîte aux lettres.
-maman|On rentre.
-papa|Le bouton tient encore, tout juste.
-narrateur|Le soir, l'écharpe sèche près du radiateur.
-narrateur|Sarah regarde la boîte aux lettres, par la porte.
-enfant-f|Le chemin est encore un peu là.
-maman|Un peu, oui.
-papa|Demain, il sera peut-être parti.
-narrateur|Sarah touche le fil du bouton.
-maman|On le recoud tout à l'heure.
-enfant-f|Le livre aussi avait un escargot.
-papa|Tout lent, comme le vrai.</t>
+          <t>narrateur|Sarah veut tout dire, d'un coup.
+narrateur|Elle tire l'album trop vite.
+narrateur|Les pages se collent un peu.
+narrateur|L'album glisse vers le banc.
+enfant-f|Ça tombe !
+narrateur|Sarah veut foncer, d'un coup.
+narrateur|Sarah refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Elle pose l'album à plat.
+narrateur|Elle écoute le coin des livres.
+narrateur|Un autre enfant feuillette, plus loin.
+narrateur|Sarah attend le silence, un instant.
+enfant-f|Je peux dire quelque chose ?
+enfant-f|Il y a un escargot, dans le livre.
+narrateur|La page sent le papier épais.
+narrateur|Le soir, la porte s'ouvre.
+maman|Te voilà, Sarah.
+papa|L'écharpe sent le savon.
+narrateur|Sarah pose le cartable contre le mur.
+enfant-f|J'ai parlé du chemin.
+enfant-f|Après le ver de terre.
+papa|Merci, Sarah.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as soif ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Sarah se desserre.
+papa|L'écharpe, tu la vois ?
+enfant-f|Oui, papa.
+narrateur|Le bois du crochet tient la laine.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>pages,porte</t>
         </is>
       </c>
     </row>
@@ -1965,17 +2022,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bouton de laine ne pend plus. Le chemin était d'argent. Bonne soirée, ma grande.</t>
+          <t>Ils s'arrêtent devant la vitre. Le chemin d'argent est plus sec. L'éclat est là, papa. Tu le vois sur le chemin ? Oui, papa. On est bien, ici. Plus tard, l'écharpe sèche près du radiateur. Ça sent le savon, un peu. Comme ce matin. Tu souffles ? Oui, papa. Sarah souffle. Le ventre est large, à sa place. On m'a entendue. On t'a entendue, Sarah. Oui, maman. Sarah pose la joue près de l'écharpe. La laine est sèche, un peu rêche. C'est chaud. Dehors, la vitre garde le chemin. L'éclat d'escargot tient sur la vitre.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bouton de laine ne pend plus. Le chemin était d'argent. Bonne soirée, ma grande.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent devant la vitre. Le chemin d'argent est plus sec. L'éclat est là, papa. Tu le vois sur le chemin ? Oui, papa. On est bien, ici. Plus tard, l'écharpe sèche près du radiateur. Ça sent le savon, un peu. Comme ce matin. Tu souffles ? Oui, papa. Sarah souffle. Le ventre est large, à sa place. On m'a entendue. On t'a entendue, Sarah. Oui, maman. Sarah pose la joue près de l'écharpe. La laine est sèche, un peu rêche. C'est chaud. Dehors, la vitre garde le chemin. L'&lt;emphasis level="moderate"&gt;éclat d'escargot&lt;/emphasis&gt; tient sur la vitre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent devant la vitre. Le chemin d'argent est plus sec. L'éclat est là, papa. Tu le vois sur le chemin ? Oui, papa. On est bien, ici. Plus tard, l'écharpe sèche près du radiateur. Ça sent le savon, un peu. Comme ce matin. Tu souffles ? Oui, papa. Sarah souffle. Le ventre est large, à sa place. On m'a entendue. On t'a entendue, Sarah. Oui, maman. Sarah pose la joue près de l'écharpe. La laine est sèche, un peu rêche. C'est chaud. Dehors, la vitre garde le chemin. L'&lt;emphasis&gt;éclat d'escargot&lt;/emphasis&gt; tient sur la vitre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2022,18 +2079,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2042,12 +2099,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2056,17 +2113,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'escargot</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2075,11 +2136,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2088,26 +2149,53 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_tient_sur_la_vitre; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bouton de laine ne pend plus.
-papa|Le chemin était d'argent.
-maman|Bonne soirée, ma grande.</t>
+          <t>narrateur|Ils s'arrêtent devant la vitre.
+narrateur|Le chemin d'argent est plus sec.
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur le chemin ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|Plus tard, l'écharpe sèche près du radiateur.
+narrateur|Ça sent le savon, un peu.
+enfant-f|Comme ce matin.
+papa|Tu souffles ?
+enfant-f|Oui, papa.
+narrateur|Sarah souffle.
+narrateur|Le ventre est large, à sa place.
+enfant-f|On m'a entendue.
+maman|On t'a entendue, Sarah.
+enfant-f|Oui, maman.
+narrateur|Sarah pose la joue près de l'écharpe.
+narrateur|La laine est sèche, un peu rêche.
+enfant-f|C'est chaud.
+narrateur|Dehors, la vitre garde le chemin.
+narrateur|L'éclat d'escargot tient sur la vitre.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radiateur,vitre</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2213,6 +2301,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>